<commit_message>
feat: XlsxAdapter v1.1 contract, update integration tests, add test data
</commit_message>
<xml_diff>
--- a/test_cpe.xlsx
+++ b/test_cpe.xlsx
@@ -413,141 +413,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>tipo_doc</t>
+          <t>cpe_tipo</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>serie</t>
+          <t>cpe_serie</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>numero</t>
+          <t>cpe_numero</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>fecha_emision</t>
+          <t>cpe_fecha</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>moneda</t>
+          <t>cli_tipo_doc</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>forma_pago</t>
+          <t>cli_num_doc</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>cliente_tipo_doc</t>
+          <t>cli_nombre</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>cliente_numero_doc</t>
+          <t>cli_direccion</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>cliente_denominacion</t>
+          <t>venta_subtotal</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>cliente_direccion</t>
+          <t>venta_igv</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>total_gravada</t>
+          <t>venta_total</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>total_exonerada</t>
+          <t>pago_forma</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>total_inafecta</t>
+          <t>estado</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>total_igv</t>
+          <t>item_orden</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>total_icbper</t>
+          <t>item_codigo</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>item_descripcion</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>item_codigo</t>
+          <t>item_unidad</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>item_descripcion</t>
+          <t>item_unspsc</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>item_unspsc</t>
+          <t>item_cantidad</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>item_unidad</t>
+          <t>item_precio_unit</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>item_cantidad</t>
+          <t>item_valor_unitario</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>item_precio_con_igv</t>
+          <t>item_descuento</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>item_precio_sin_igv</t>
+          <t>item_subtotal_sin_igv</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>item_subtotal_sin_igv</t>
+          <t>item_igv</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>item_igv</t>
+          <t>item_total</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
-        <is>
-          <t>item_total</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
         <is>
           <t>item_afectacion_igv</t>
         </is>
@@ -564,103 +559,320 @@
           <t>B001</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>100</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>00000100</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>18-04-2026</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PEN</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Contado</t>
+          <t>00000000</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>CLIENTES VARIOS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>00000000</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>CLIENTE VARIOS</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I2" t="n">
+        <v>16.949</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3.051</v>
       </c>
       <c r="K2" t="n">
-        <v>16.95</v>
-      </c>
-      <c r="L2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>EFECTIVO</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>BORRADOR</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>PARACETAMOL 500MG X 10</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>NIU</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>10000000</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2" t="n">
+        <v>10</v>
+      </c>
+      <c r="U2" t="n">
+        <v>8.474600000000001</v>
+      </c>
+      <c r="V2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
+      <c r="W2" t="n">
+        <v>16.949</v>
+      </c>
+      <c r="X2" t="n">
+        <v>3.051</v>
+      </c>
+      <c r="Y2" t="n">
         <v>20</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00000101</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>00000000</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CLIENTES VARIOS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>YAPE</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>BORRADOR</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>AGUA OXIGENADA 120ML</t>
+        </is>
+      </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>NIU</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>PRODUCTO TEST</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
           <t>10000000</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="S3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" t="n">
+        <v>6</v>
+      </c>
+      <c r="U3" t="n">
+        <v>6</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>6</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>00000011</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>20100070970</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>EMPRESA EJEMPLO S.A.C.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>AV. LIMA 123</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="n">
+        <v>18</v>
+      </c>
+      <c r="K4" t="n">
+        <v>118</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>BORRADOR</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>AMOXICILINA 500MG X 21</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>NIU</t>
         </is>
       </c>
-      <c r="U3" t="n">
-        <v>1</v>
-      </c>
-      <c r="V3" t="n">
-        <v>20</v>
-      </c>
-      <c r="W3" t="n">
-        <v>16.95</v>
-      </c>
-      <c r="X3" t="n">
-        <v>16.95</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>20</v>
-      </c>
-      <c r="AA3" t="inlineStr">
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>10000000</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T4" t="n">
+        <v>59</v>
+      </c>
+      <c r="U4" t="n">
+        <v>50</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>100</v>
+      </c>
+      <c r="X4" t="n">
+        <v>18</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>118</v>
+      </c>
+      <c r="Z4" t="inlineStr">
         <is>
           <t>10</t>
         </is>

</xml_diff>